<commit_message>
Track retest results for questions 3.2 and 3.3
3.2 (confirmed pilot error, И-12-10-03): partially improved -- source now connected, printed-pick-list branch addressed, but the exact "перепровести Заявку на комплектацию" instruction from the error analysis is still not given.
3.3 (was already correct, not an error): unchanged and correct, with more procedural detail than the original pilot answer.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DpSN8JwCJ3tg3JVUadr2zE
</commit_message>
<xml_diff>
--- a/docs/accounts/eco/pilot-test-02-retest.xlsx
+++ b/docs/accounts/eco/pilot-test-02-retest.xlsx
@@ -902,12 +902,24 @@
           <t>Корректировка заказа описана, но ситуация с распечатанной заявкой не закрыта.</t>
         </is>
       </c>
-      <c r="J9" s="14" t="n"/>
-      <c r="K9" s="14" t="n"/>
-      <c r="L9" s="14" t="n"/>
-      <c r="M9" s="32" t="inlineStr">
-        <is>
-          <t>Не перепроверено</t>
+      <c r="J9" s="33" t="inlineStr">
+        <is>
+          <t>12.09.2026</t>
+        </is>
+      </c>
+      <c r="K9" s="33" t="inlineStr">
+        <is>
+          <t>1. Откройте оформленный Заказ и создайте к нему корректировку. 2. В корректировке удалите строку с прежней характеристикой товара и новой строкой добавьте ту же номенклатуру с требуемой характеристикой. 3. Поскольку заявка на сборку уже распечатана, проверьте, сформирован ли по заказу Заказ на производство: если да, для изменения продукта обратитесь к ОБ.</t>
+        </is>
+      </c>
+      <c r="L9" s="33" t="inlineStr">
+        <is>
+          <t>И-12-10-03 «Корректировка Заказу покупателя в 1С».docx — 64% (в исходном пилоте этот источник числился как «не загружен в корпус» — теперь есть и цитируется).</t>
+        </is>
+      </c>
+      <c r="M9" s="33" t="inlineStr">
+        <is>
+          <t>ЧАСТИЧНО УЛУЧШЕНО — источник наконец подключён и появился шаг именно про распечатанную заявку, но конкретная инструкция «перепровести Заявку на комплектацию» (из разбора ошибок) всё ещё не дана — только условный переход «если сформирован Заказ на производство → к ОБ»</t>
         </is>
       </c>
     </row>
@@ -938,12 +950,24 @@
           <t>Подробно расписаны роли, документы и дальнейшие ветки процесса.</t>
         </is>
       </c>
-      <c r="J10" s="14" t="n"/>
-      <c r="K10" s="14" t="n"/>
-      <c r="L10" s="14" t="n"/>
+      <c r="J10" s="14" t="inlineStr">
+        <is>
+          <t>12.09.2026</t>
+        </is>
+      </c>
+      <c r="K10" s="14" t="inlineStr">
+        <is>
+          <t>5-шаговый процесс: решение руководителя ОКК/директора по качеству (Акт забраковки ТМЦ, форма 03-01); действия сотрудника ОКК (письмо, Акт разрешения на отклонение, Журнал форма 03-03); отдельная ветка для опасного брака/аллергенов; роли ведущего технолога ПО/НА/ОИМРП/начальника ЛР; хранение и дальнейшие действия по браку.</t>
+        </is>
+      </c>
+      <c r="L10" s="14" t="inlineStr">
+        <is>
+          <t>ПР-03-00-12.doc — 62%; ПР-08-00-14 упомянут в тексте.</t>
+        </is>
+      </c>
       <c r="M10" s="32" t="inlineStr">
         <is>
-          <t>Не перепроверено</t>
+          <t>БЕЗ ИЗМЕНЕНИЙ (было верно, осталось верно) — ответ даже детальнее исходного (названы конкретные формы 03-01/03-03 и роли, которых не было в версии от 11.09)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Track retest result for question 4.1 (unchanged, correctly reports no data)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DpSN8JwCJ3tg3JVUadr2zE
</commit_message>
<xml_diff>
--- a/docs/accounts/eco/pilot-test-02-retest.xlsx
+++ b/docs/accounts/eco/pilot-test-02-retest.xlsx
@@ -998,12 +998,24 @@
           <t>Запрошенная марка не найдена.</t>
         </is>
       </c>
-      <c r="J11" s="14" t="n"/>
-      <c r="K11" s="14" t="n"/>
-      <c r="L11" s="14" t="n"/>
+      <c r="J11" s="14" t="inlineStr">
+        <is>
+          <t>12.09.2026</t>
+        </is>
+      </c>
+      <c r="K11" s="14" t="inlineStr">
+        <is>
+          <t>В доступных источниках марка стретч-плёнки для обмотки паллет с готовой продукцией не указана. Найденный фрагмент Д-09-01-17 «План контроля тары и упаковки» содержит требования к пакетам и этикеткам, но не к стретч-плёнке.</t>
+        </is>
+      </c>
+      <c r="L11" s="14" t="inlineStr">
+        <is>
+          <t>Д-09-01-17 План контроля тары и упаковки.docx — 50%</t>
+        </is>
+      </c>
       <c r="M11" s="32" t="inlineStr">
         <is>
-          <t>Не перепроверено</t>
+          <t>БЕЗ ИЗМЕНЕНИЙ — верный ответ «не найдено» (уже подтверждено в pilot-test-01-analysis.md §5: марки в корпусе действительно нет)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Track retest result for question 4.2 (still open, closer but no periodicity found)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DpSN8JwCJ3tg3JVUadr2zE
</commit_message>
<xml_diff>
--- a/docs/accounts/eco/pilot-test-02-retest.xlsx
+++ b/docs/accounts/eco/pilot-test-02-retest.xlsx
@@ -1046,12 +1046,24 @@
           <t>Нет конкретной периодичности.</t>
         </is>
       </c>
-      <c r="J12" s="14" t="n"/>
-      <c r="K12" s="14" t="n"/>
-      <c r="L12" s="14" t="n"/>
+      <c r="J12" s="14" t="inlineStr">
+        <is>
+          <t>12.09.2026</t>
+        </is>
+      </c>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>В доступных источниках периодичность оценки квалификации внештатных сотрудников, работающих по договору подряда, не указана. В ПР-14-00-12 «Компетентность персонала» найдено поле «Оценка результативности», но срок или частота такой оценки не приведены.</t>
+        </is>
+      </c>
+      <c r="L12" s="14" t="inlineStr">
+        <is>
+          <t>Д-17-12-03 Оборудование для мониторинга и измерений.docx — 48%; ПР-14-00-12 Компетентность персонала.doc — 48%</t>
+        </is>
+      </c>
       <c r="M12" s="32" t="inlineStr">
         <is>
-          <t>Не перепроверено</t>
+          <t>БЕЗ ИЗМЕНЕНИЙ — вопрос остаётся открытым (был не подтверждён ни как ошибка, ни как верный ответ в pilot-test-01-analysis.md §5). Теперь хотя бы нашли релевантное поле «Оценка результативности» в ПР-14-00-12, но конкретики по подрядчикам по-прежнему нет — похоже, нужного документа/раздела действительно нет в корпусе.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Track retest result for question 4.3 (unchanged, correctly reports no data)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DpSN8JwCJ3tg3JVUadr2zE
</commit_message>
<xml_diff>
--- a/docs/accounts/eco/pilot-test-02-retest.xlsx
+++ b/docs/accounts/eco/pilot-test-02-retest.xlsx
@@ -1094,12 +1094,24 @@
           <t>Перечень требуемых полей отсутствует.</t>
         </is>
       </c>
-      <c r="J13" s="14" t="n"/>
-      <c r="K13" s="14" t="n"/>
-      <c r="L13" s="14" t="n"/>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>12.09.2026</t>
+        </is>
+      </c>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>В найденных источниках точный перечень полей журнала «Учёт уборки производственного оборудования», форма 17-08, не указан. Найден только перечень полей для журнала оборудования для мониторинга и измерений (другая форма): наименование оборудования и номер, дата последней поверки, подпись ответственного, дата следующей поверки, подпись ответственного, место установки, примечание.</t>
+        </is>
+      </c>
+      <c r="L13" s="14" t="inlineStr">
+        <is>
+          <t>Д-17-12-03 «Оборудование для мониторинга и измерений».docx — 75% (другой документ, не тот, что цитировался в пилоте — но вывод тот же: нужного перечня нет)</t>
+        </is>
+      </c>
       <c r="M13" s="32" t="inlineStr">
         <is>
-          <t>Не перепроверено</t>
+          <t>БЕЗ ИЗМЕНЕНИЙ — верный ответ «не найдено» (Форма 17-08 как бланк по-прежнему не в корпусе, см. pilot-test-01-analysis.md §5). Источник цитирования сменился на другой документ — не тот, что раньше, но конечный вывод не изменился.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Track retest result for question 5.1 (improved -- was open, now full direct answer)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DpSN8JwCJ3tg3JVUadr2zE
</commit_message>
<xml_diff>
--- a/docs/accounts/eco/pilot-test-02-retest.xlsx
+++ b/docs/accounts/eco/pilot-test-02-retest.xlsx
@@ -24,7 +24,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -61,6 +61,11 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border/>
@@ -69,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -146,6 +151,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1142,12 +1150,24 @@
           <t>Объяснено условие и дальнейший путь, но прямой алгоритм для заданной ситуации отсутствует.</t>
         </is>
       </c>
-      <c r="J14" s="14" t="n"/>
-      <c r="K14" s="14" t="n"/>
-      <c r="L14" s="14" t="n"/>
-      <c r="M14" s="32" t="inlineStr">
-        <is>
-          <t>Не перепроверено</t>
+      <c r="J14" s="34" t="inlineStr">
+        <is>
+          <t>12.09.2026</t>
+        </is>
+      </c>
+      <c r="K14" s="34" t="inlineStr">
+        <is>
+          <t>1. Дождитесь уведомления ОКК о соответствии сырья требованиям. 2. ОКК направляет письмо руководителю ОКК, бухгалтерии, начальнику СО и оператору склада с просьбой переместить сырьё на соответствующий склад. 3. После перемещения на рабочий склад согласуйте с мастером ПО приоритетность задач. 4. В 1С8 во вкладке «Процесс» заказа установите флажок «Передать сырьё» и нажмите «Выгрузить WMS». 5. После выдачи оператор ПО забирает сырьё и доставляет к указанному аппарату.</t>
+        </is>
+      </c>
+      <c r="L14" s="34" t="inlineStr">
+        <is>
+          <t>ПР-09-00-14 «Контроль качества».doc — 49%; ПР-03-00-12.doc — 65%; Д-08-07-01 упомянут в тексте</t>
+        </is>
+      </c>
+      <c r="M14" s="34" t="inlineStr">
+        <is>
+          <t>УЛУЧШЕНО — раньше был открытый вопрос («прямого порядка... нет»), теперь дан полный прямой пошаговый ответ именно для склада «Проверка ОКК», с конкретным источником (ПР-09-00-14), который мы раньше не связывали с этим вопросом</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Track retest result for question 5.2 (unchanged, confirms retrieval root cause #2)
Confirms the proverka-zdorovya-zagruzki-predlozhenie.md hypothesis: this is a retrieval-layer failure, not a parsing failure (source is readable .docx with the answer present as plain text), so the fixes that resolved 1.2/1.3 (both .doc parsing issues) did not touch it -- exactly as predicted.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DpSN8JwCJ3tg3JVUadr2zE
</commit_message>
<xml_diff>
--- a/docs/accounts/eco/pilot-test-02-retest.xlsx
+++ b/docs/accounts/eco/pilot-test-02-retest.xlsx
@@ -1198,12 +1198,24 @@
           <t>Есть правило только для одного типа аварий, но нет общего ранжирования заявок.</t>
         </is>
       </c>
-      <c r="J15" s="14" t="n"/>
-      <c r="K15" s="14" t="n"/>
-      <c r="L15" s="14" t="n"/>
-      <c r="M15" s="32" t="inlineStr">
-        <is>
-          <t>Не перепроверено</t>
+      <c r="J15" s="33" t="inlineStr">
+        <is>
+          <t>12.09.2026</t>
+        </is>
+      </c>
+      <c r="K15" s="33" t="inlineStr">
+        <is>
+          <t>В доступных источниках не найден порядок приоритизации нескольких срочных заявок на ремонт. Поэтому определить, какую заявку выполнять первой, по имеющимся данным нельзя.</t>
+        </is>
+      </c>
+      <c r="L15" s="33" t="inlineStr">
+        <is>
+          <t>Источник не показан вообще (карточка «Ответ основан на источниках» отсутствует в ответе)</t>
+        </is>
+      </c>
+      <c r="M15" s="33" t="inlineStr">
+        <is>
+          <t>БЕЗ ИЗМЕНЕНИЙ — важное подтверждение гипотезы «Корневая причина №2» из proverka-zdorovya-zagruzki-predlozhenie.md: это retrieval-ошибка, не парсинг (источник ПР-10(02)-00.docx читаемый, ответ в нём есть текстом), и правки, починившие 1.2/1.3, её не задели — ровно как предсказывалось</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Track retest result for question 5.3 (unchanged, correct, more detailed)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DpSN8JwCJ3tg3JVUadr2zE
</commit_message>
<xml_diff>
--- a/docs/accounts/eco/pilot-test-02-retest.xlsx
+++ b/docs/accounts/eco/pilot-test-02-retest.xlsx
@@ -1246,12 +1246,24 @@
           <t>Дан практический алгоритм с учётом приоритетов и действий в 1С.</t>
         </is>
       </c>
-      <c r="J16" s="14" t="n"/>
-      <c r="K16" s="14" t="n"/>
-      <c r="L16" s="14" t="n"/>
+      <c r="J16" s="14" t="inlineStr">
+        <is>
+          <t>12.09.2026</t>
+        </is>
+      </c>
+      <c r="K16" s="14" t="inlineStr">
+        <is>
+          <t>Срочный заказ покупателя имеет приоритет над наработкой продукции на склад (если у заказа нет поля «Приоритет» или указан «0», выполняется после заказов «1»/«2»). Порядок: 1) через отчёт «Загруженность оборудования» определить окно; 2) согласовать график наработки с мастером ПО/техдиректором/начальником ПУ; 3) сформировать заказ на производство на доп. объём без привязки к заказу покупателя; 4) проверить складские остатки аналогичной продукции.</t>
+        </is>
+      </c>
+      <c r="L16" s="14" t="inlineStr">
+        <is>
+          <t>И-12-10-03.docx 63%; ПР-08-00-14.doc 49%; Д-08-03-01.doc 49%; И-08-08-01.docx 48% — все релевантны, аномалий нет</t>
+        </is>
+      </c>
       <c r="M16" s="32" t="inlineStr">
         <is>
-          <t>Не перепроверено</t>
+          <t>БЕЗ ИЗМЕНЕНИЙ (было верно, осталось верно) — не входил в число ошибок пилота; ответ даже детальнее, с постатейной сверкой источников</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add test conditions section and full sync of retest protocol (17/18 done)
Added a critical "Условия проведения" section capturing model (OpenAI/gpt-5.5), agent mode, reasoning-off setting, and search scope (Данные+Документы, narrowed to the ЭКО collection) from the live UI screenshot -- flagged as an open question whether these matched the original 11.09 pilot's conditions, since a mismatch could explain some of the observed changes independent of any corpus/parser fix.

Rewrote the .md wholesale to stay in sync with the .docx after many incremental edits. Current tally at 17/18 retested: 3 fixed (1.2, 1.3, 5.1), 1 partially improved (3.2), 1 regression (2.1), 3 unchanged-still-broken (2.2, 2.3, 5.2 -- the last confirming the retrieval root-cause-2 hypothesis), 7 unchanged-correct, 1 remaining (6.3; 6.2 also still pending in the sheet).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DpSN8JwCJ3tg3JVUadr2zE
</commit_message>
<xml_diff>
--- a/docs/accounts/eco/pilot-test-02-retest.xlsx
+++ b/docs/accounts/eco/pilot-test-02-retest.xlsx
@@ -1294,12 +1294,24 @@
           <t>Полный алгоритм до и после фасовки.</t>
         </is>
       </c>
-      <c r="J17" s="14" t="n"/>
-      <c r="K17" s="14" t="n"/>
-      <c r="L17" s="14" t="n"/>
+      <c r="J17" s="14" t="inlineStr">
+        <is>
+          <t>12.09.2026</t>
+        </is>
+      </c>
+      <c r="K17" s="14" t="inlineStr">
+        <is>
+          <t>1. Перед началом проверяет в Рабочей инструкции на производство (форма 16-03): примечания к технологическому процессу, вид фасовки. 2. Осматривает тару и упаковку. 3. Выполняет фасовку по И-08-02 «Фасовка и упаковка готовой продукции». 4. После каждого этапа — запись и подпись. 5. Вывозит продукцию в зону передачи на склад. 6. Передаёт заполненную рабочую инструкцию ответственному сотруднику ПО. Фасовке подлежит продукция с положительным заключением ОКК либо продукция, предназначенная для перефасовки.</t>
+        </is>
+      </c>
+      <c r="L17" s="14" t="inlineStr">
+        <is>
+          <t>ПР-08-00-14 «Производственный процесс», разделы 5.4-5.7.doc — 57%; И-08-02-10 «Фасовка и упаковка готовой продукции».doc — 50%</t>
+        </is>
+      </c>
       <c r="M17" s="32" t="inlineStr">
         <is>
-          <t>Не перепроверено</t>
+          <t>БЕЗ ИЗМЕНЕНИЙ (было верно, осталось верно) — не входил в число ошибок пилота, ответ детальнее исходного</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Track retest result for question 6.2 (service error both attempts, wrong sources retrieved)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DpSN8JwCJ3tg3JVUadr2zE
</commit_message>
<xml_diff>
--- a/docs/accounts/eco/pilot-test-02-retest.xlsx
+++ b/docs/accounts/eco/pilot-test-02-retest.xlsx
@@ -24,7 +24,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +66,11 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border/>
@@ -74,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -154,6 +159,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1342,12 +1350,24 @@
           <t>Дан процесс запроса, но не инструкция по добавлению в 1С.</t>
         </is>
       </c>
-      <c r="J18" s="14" t="n"/>
-      <c r="K18" s="14" t="n"/>
-      <c r="L18" s="14" t="n"/>
-      <c r="M18" s="32" t="inlineStr">
-        <is>
-          <t>Не перепроверено</t>
+      <c r="J18" s="35" t="inlineStr">
+        <is>
+          <t>12.09.2026</t>
+        </is>
+      </c>
+      <c r="K18" s="35" t="inlineStr">
+        <is>
+          <t>ОШИБКА СЕРВИСА (дважды подряд, 13:50 и 13:51): «Не удалось получить ответ модели (временная ошибка сервиса). Попробуйте повторить запрос или переформулировать короче.» Содержательного ответа нет ни разу.</t>
+        </is>
+      </c>
+      <c r="L18" s="35" t="inlineStr">
+        <is>
+          <t>Даже при отказе модели показаны источники — но НЕ те: Д-08-03-01 «Формирование заказов на производство» (63-64%) и Д-08-04-01 «Проведение корректировок к заказу на производство» (59-61%). Ни разу не показан И-08-05-08 «Внесение спецификаций в базе 1С-8» — реальный нужный источник по разбору ошибок пилота.</t>
+        </is>
+      </c>
+      <c r="M18" s="35" t="inlineStr">
+        <is>
+          <t>НЕ ОЦЕНИВАЕТСЯ — служебная ошибка модели, а не содержательный ответ. Отдельно тревожно: retrieval даже не подтягивает нужный документ (И-08-05-08) — похоже на путаницу с похожими по теме документами «заказ на производство», а не на восстановленный/сломанный формат</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Finalize retest protocol -- all 18/18 questions retested
Final tally: 3 fixed (1.2, 1.3, 5.1), 1 partially improved (3.2), 1 regression (2.1), 4 unchanged-still-broken (2.2, 2.3, 5.2, 6.2 -- the last a service error with wrong-document retrieval on top), 9 unchanged-correct. Of the original 7 confirmed pilot errors: 3 fixed, 1 partial, 3 still broken. 5.2 confirms the retrieval root-cause-2 hypothesis exactly as predicted (readable source, answer present as text, still not found). Flagged a citation-integrity pattern (2 consecutive answers cited a UI source file unrelated to the answer text) as a priority to investigate before any corpus cleanup.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DpSN8JwCJ3tg3JVUadr2zE
</commit_message>
<xml_diff>
--- a/docs/accounts/eco/pilot-test-02-retest.xlsx
+++ b/docs/accounts/eco/pilot-test-02-retest.xlsx
@@ -1398,12 +1398,24 @@
           <t>Последовательно описаны этапы, сроки, фиксация и действия при несоответствии.</t>
         </is>
       </c>
-      <c r="J19" s="14" t="n"/>
-      <c r="K19" s="14" t="n"/>
-      <c r="L19" s="14" t="n"/>
+      <c r="J19" s="14" t="inlineStr">
+        <is>
+          <t>12.09.2026</t>
+        </is>
+      </c>
+      <c r="K19" s="14" t="inlineStr">
+        <is>
+          <t>Процесс установлен документом ПР-09-00 «Контроль качества»: 1) контроль на складе сырья СО или в ОКК; 2) результаты в журнал «Контроль сырья и первичной упаковки» (форма 09-01) с полным перечнем полей; 3) при несоответствии решение принимает руководитель ОКК/директор по качеству; 4) оформляются Акт забраковки (03-01)/Акт разрешения на отклонение (03-02)/Акт на утилизацию (03-04), запись в журнал 03-03; 5) решение о применении сырья и коррекции — руководитель/директор по качеству.</t>
+        </is>
+      </c>
+      <c r="L19" s="14" t="inlineStr">
+        <is>
+          <t>ПР-09-00-14 «Контроль качества».doc — 63%; ПР-03-00-12 упомянут в тексте</t>
+        </is>
+      </c>
       <c r="M19" s="32" t="inlineStr">
         <is>
-          <t>Не перепроверено</t>
+          <t>БЕЗ ИЗМЕНЕНИЙ (было верно, осталось верно) — не входил в число ошибок пилота, ответ детальнее исходного (конкретные формы 09-01/03-01/03-02/03-03/03-04)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add было→стало summary table and time column to retest protocol
Adds a consolidated "было (11.09) → стало (12.09)" overview table
covering all 18 questions to the retest protocol (md/docx), plus an
explicit "Дата и время" row in the test-conditions table noting the
single known timestamp range (13:44-13:46) with no per-question times
available.

In the tracking spreadsheet, adds a "Время" column carrying that same
range, and a new "Категория" column (Исправлено/Регрессия/Без
изменений и т.д.) colored per the existing green/yellow/red/grey
legend for at-a-glance scanning.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DpSN8JwCJ3tg3JVUadr2zE
</commit_message>
<xml_diff>
--- a/docs/accounts/eco/pilot-test-02-retest.xlsx
+++ b/docs/accounts/eco/pilot-test-02-retest.xlsx
@@ -12,7 +12,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -23,8 +23,14 @@
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Carlito"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -71,6 +77,26 @@
         <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E1D5F0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border/>
@@ -79,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -162,6 +188,18 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -450,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -462,9 +500,11 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="28" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="55" customWidth="1" min="11" max="11"/>
-    <col width="40" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="34" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -509,19 +549,29 @@
           <t>Дата ре-теста</t>
         </is>
       </c>
-      <c r="K1" s="31" t="inlineStr">
+      <c r="K1" s="36" t="inlineStr">
+        <is>
+          <t>Время (диапазон теста)</t>
+        </is>
+      </c>
+      <c r="L1" s="31" t="inlineStr">
         <is>
           <t>Ответ при ре-тесте (12.09.2026)</t>
         </is>
       </c>
-      <c r="L1" s="31" t="inlineStr">
+      <c r="M1" s="31" t="inlineStr">
         <is>
           <t>Источник(и) при ре-тесте</t>
         </is>
       </c>
-      <c r="M1" s="31" t="inlineStr">
+      <c r="N1" s="31" t="inlineStr">
         <is>
           <t>Статус ре-теста</t>
+        </is>
+      </c>
+      <c r="O1" s="36" t="inlineStr">
+        <is>
+          <t>Категория (сводно, см. §7 протокола)</t>
         </is>
       </c>
     </row>
@@ -569,17 +619,27 @@
       </c>
       <c r="K2" s="14" t="inlineStr">
         <is>
+          <t>13:44–13:46 (единый диапазон по скриншоту условий теста; отдельных отметок времени на вопрос нет)</t>
+        </is>
+      </c>
+      <c r="L2" s="14" t="inlineStr">
+        <is>
           <t>Организовать маркировку несоответствующих ТМЦ этим актом (упакованную паллету допускается маркировать четырьмя экземплярами акта — по одному с каждой стороны); переместить ТМЦ в зону «БРАК» не позднее 1 рабочего дня; разместить по требованиям акта; согласовать с бухгалтером по учёту ТМЦ перемещение в 1С-8 на склад «БРАК».</t>
         </is>
       </c>
-      <c r="L2" s="14" t="inlineStr">
+      <c r="M2" s="14" t="inlineStr">
         <is>
           <t>ПР-03-00-12 Несоответствующая продукция.doc — 60%</t>
         </is>
       </c>
-      <c r="M2" s="14" t="inlineStr">
+      <c r="N2" s="14" t="inlineStr">
         <is>
           <t>Без изменений (уже был верным)</t>
+        </is>
+      </c>
+      <c r="O2" s="37" t="inlineStr">
+        <is>
+          <t>Без изменений — верно</t>
         </is>
       </c>
     </row>
@@ -627,17 +687,27 @@
       </c>
       <c r="K3" s="16" t="inlineStr">
         <is>
+          <t>13:44–13:46 (единый диапазон по скриншоту условий теста; отдельных отметок времени на вопрос нет)</t>
+        </is>
+      </c>
+      <c r="L3" s="16" t="inlineStr">
+        <is>
           <t>Экспериментальной выработкой руководит технолог лаборатории: он управляет производственным процессом и при необходимости вносит корректировки в технологию с отражением их в РИ (Форма 16-03). После завершения процесса образец передают в ОКК; при отклонении качества продукт дорабатывается под руководством технолога лаборатории.</t>
         </is>
       </c>
-      <c r="L3" s="16" t="inlineStr">
+      <c r="M3" s="16" t="inlineStr">
         <is>
           <t>ПР-03-00-12 Несоответствующая продукция.doc — 53%; И-16-01-11 Внедрение новых видов продукции в производство.doc — 41%</t>
         </is>
       </c>
-      <c r="M3" s="16" t="inlineStr">
+      <c r="N3" s="16" t="inlineStr">
         <is>
           <t>ИСПРАВЛЕНО ✅</t>
+        </is>
+      </c>
+      <c r="O3" s="34" t="inlineStr">
+        <is>
+          <t>Исправлено</t>
         </is>
       </c>
     </row>
@@ -685,17 +755,27 @@
       </c>
       <c r="K4" s="16" t="inlineStr">
         <is>
+          <t>13:44–13:46 (единый диапазон по скриншоту условий теста; отдельных отметок времени на вопрос нет)</t>
+        </is>
+      </c>
+      <c r="L4" s="16" t="inlineStr">
+        <is>
           <t>При пометке «Экспериментальная» выполняйте выработку по указаниям технолога лаборатории — он руководит экспериментальным производственным процессом и при необходимости корректирует технологию. Самостоятельно менять технологию не следует; изменения должны быть отражены в РИ (Форма 16-03). После завершения образец передают в ОКК.</t>
         </is>
       </c>
-      <c r="L4" s="16" t="inlineStr">
+      <c r="M4" s="16" t="inlineStr">
         <is>
           <t>И-09-08-02 Порядок перемещения ТМЦ с истекающим сроком хранения.doc — 61%; И-16-01-11 Внедрение новых видов продукции в производство.doc — 60%; И-15-06-08 Документальное оформление продукции ОСиС.docx — 57%; И-08-02-10 Фасовка и упаковка готовой продукции.doc — 56%</t>
         </is>
       </c>
-      <c r="M4" s="16" t="inlineStr">
+      <c r="N4" s="16" t="inlineStr">
         <is>
           <t>ИСПРАВЛЕНО ✅</t>
+        </is>
+      </c>
+      <c r="O4" s="34" t="inlineStr">
+        <is>
+          <t>Исправлено</t>
         </is>
       </c>
     </row>
@@ -733,17 +813,27 @@
       </c>
       <c r="K5" s="18" t="inlineStr">
         <is>
+          <t>13:44–13:46 (единый диапазон по скриншоту условий теста; отдельных отметок времени на вопрос нет)</t>
+        </is>
+      </c>
+      <c r="L5" s="18" t="inlineStr">
+        <is>
           <t>Какие именно поля оператор заполняет после фасовки, в найденном фрагменте не указано. Названы только поля, которые оператор проверяет ДО фасовки: «Примечания к технологическому процессу» и «Вид фасовки».</t>
         </is>
       </c>
-      <c r="L5" s="18" t="inlineStr">
+      <c r="M5" s="18" t="inlineStr">
         <is>
           <t>Текст ответа ссылается на И-08-02-10 «Фасовка и упаковка готовой продукции», раздел 3.1, и ПР-08-00-14 «Производственный процесс», раздел 5.6 — но карточка источника в чате показывает СОВСЕМ ДРУГОЙ файл: "Datafortest07.07.xlsx" (64%), не входящий в известный корпус СМК.</t>
         </is>
       </c>
-      <c r="M5" s="18" t="inlineStr">
+      <c r="N5" s="18" t="inlineStr">
         <is>
           <t>РЕГРЕССИЯ ⚠️ — было верно, стало «не найдено» + подозрительный источник</t>
+        </is>
+      </c>
+      <c r="O5" s="35" t="inlineStr">
+        <is>
+          <t>Регрессия</t>
         </is>
       </c>
     </row>
@@ -781,17 +871,27 @@
       </c>
       <c r="K6" s="33" t="inlineStr">
         <is>
+          <t>13:44–13:46 (единый диапазон по скриншоту условий теста; отдельных отметок времени на вопрос нет)</t>
+        </is>
+      </c>
+      <c r="L6" s="33" t="inlineStr">
+        <is>
           <t>При выпуске продукции с меньшим весом: 1. Откройте Заказ и создайте к нему корректировку. 2. Укажите уменьшение количества продукции — разницу со знаком «−». 3. Если по этому заказу уже есть Заказ на производство, для изменения продукта обратитесь к ОБ.</t>
         </is>
       </c>
-      <c r="L6" s="33" t="inlineStr">
+      <c r="M6" s="33" t="inlineStr">
         <is>
           <t>И-12-10-03 «Корректировка Заказу покупателя в 1С».docx — 72% (документ, который мы считали не загруженным в наш корпус — оказывается уже есть на платформе). Д-08-04-01 (реальный источник с п. 3.5.1–3.5.5) по-прежнему НЕ цитируется.</t>
         </is>
       </c>
-      <c r="M6" s="33" t="inlineStr">
+      <c r="N6" s="33" t="inlineStr">
         <is>
           <t>БЕЗ ИЗМЕНЕНИЙ — ошибка сохраняется, тот же общий ответ про Заказ покупателя вместо конкретной процедуры для Заказа на производство</t>
+        </is>
+      </c>
+      <c r="O6" s="35" t="inlineStr">
+        <is>
+          <t>Без изменений — ошибка сохраняется</t>
         </is>
       </c>
     </row>
@@ -829,17 +929,27 @@
       </c>
       <c r="K7" s="33" t="inlineStr">
         <is>
+          <t>13:44–13:46 (единый диапазон по скриншоту условий теста; отдельных отметок времени на вопрос нет)</t>
+        </is>
+      </c>
+      <c r="L7" s="33" t="inlineStr">
+        <is>
           <t>В доступном фрагменте высота сбрасывания не указана. Для канистры объёмом 5 л установлено: одно падение на дно без разрушения и течи; методика — № 38, запись выполняется в форме 09-01. Источник (по тексту): Д-09-01-17 «План контроля тары и упаковки».</t>
         </is>
       </c>
-      <c r="L7" s="33" t="inlineStr">
+      <c r="M7" s="33" t="inlineStr">
         <is>
           <t>Карточка источника показывает файл "глоссарий" (100%) — не совпадает с названным в тексте Д-09-01-17. Нужная цифра (0,8 м для диапазона 1,5–5,0 л) по-прежнему не дана, хотя она есть в Методике №38, Таблица 2 (подтверждено нами через catdoc).</t>
         </is>
       </c>
-      <c r="M7" s="33" t="inlineStr">
+      <c r="N7" s="33" t="inlineStr">
         <is>
           <t>БЕЗ ИЗМЕНЕНИЙ — тот же пробел, + вторая аномалия цитирования (после 2.1) — источник в карточке не совпадает с названным в тексте</t>
+        </is>
+      </c>
+      <c r="O7" s="35" t="inlineStr">
+        <is>
+          <t>Без изменений — ошибка сохраняется</t>
         </is>
       </c>
     </row>
@@ -877,17 +987,27 @@
       </c>
       <c r="K8" s="14" t="inlineStr">
         <is>
+          <t>13:44–13:46 (единый диапазон по скриншоту условий теста; отдельных отметок времени на вопрос нет)</t>
+        </is>
+      </c>
+      <c r="L8" s="14" t="inlineStr">
+        <is>
           <t>Согласовывает с мастером ПО приоритетность задач на день; в 1С8 во вкладке «Процесс» устанавливает флажок «Передать сырьё» и нажимает «Выгрузить WMS»; при отсутствии отметки «Подбор сырья завершён» связывается с СО; после выдачи забирает сырьё и подвозит к аппарату.</t>
         </is>
       </c>
-      <c r="L8" s="14" t="inlineStr">
+      <c r="M8" s="14" t="inlineStr">
         <is>
           <t>И-15-06-08.docx 61%; И-08-03-09.doc 59%; ПР-08-00-14.doc 48%; И-16-01-11.doc 46%; Д-08-07-01.doc 46% — все релевантны, аномалий цитирования нет.</t>
         </is>
       </c>
-      <c r="M8" s="32" t="inlineStr">
+      <c r="N8" s="32" t="inlineStr">
         <is>
           <t>БЕЗ ИЗМЕНЕНИЙ (было верно, осталось верно) — не входил в число ошибок пилота</t>
+        </is>
+      </c>
+      <c r="O8" s="37" t="inlineStr">
+        <is>
+          <t>Без изменений — верно</t>
         </is>
       </c>
     </row>
@@ -925,17 +1045,27 @@
       </c>
       <c r="K9" s="33" t="inlineStr">
         <is>
+          <t>13:44–13:46 (единый диапазон по скриншоту условий теста; отдельных отметок времени на вопрос нет)</t>
+        </is>
+      </c>
+      <c r="L9" s="33" t="inlineStr">
+        <is>
           <t>1. Откройте оформленный Заказ и создайте к нему корректировку. 2. В корректировке удалите строку с прежней характеристикой товара и новой строкой добавьте ту же номенклатуру с требуемой характеристикой. 3. Поскольку заявка на сборку уже распечатана, проверьте, сформирован ли по заказу Заказ на производство: если да, для изменения продукта обратитесь к ОБ.</t>
         </is>
       </c>
-      <c r="L9" s="33" t="inlineStr">
+      <c r="M9" s="33" t="inlineStr">
         <is>
           <t>И-12-10-03 «Корректировка Заказу покупателя в 1С».docx — 64% (в исходном пилоте этот источник числился как «не загружен в корпус» — теперь есть и цитируется).</t>
         </is>
       </c>
-      <c r="M9" s="33" t="inlineStr">
+      <c r="N9" s="33" t="inlineStr">
         <is>
           <t>ЧАСТИЧНО УЛУЧШЕНО — источник наконец подключён и появился шаг именно про распечатанную заявку, но конкретная инструкция «перепровести Заявку на комплектацию» (из разбора ошибок) всё ещё не дана — только условный переход «если сформирован Заказ на производство → к ОБ»</t>
+        </is>
+      </c>
+      <c r="O9" s="38" t="inlineStr">
+        <is>
+          <t>Частично улучшено</t>
         </is>
       </c>
     </row>
@@ -973,17 +1103,27 @@
       </c>
       <c r="K10" s="14" t="inlineStr">
         <is>
+          <t>13:44–13:46 (единый диапазон по скриншоту условий теста; отдельных отметок времени на вопрос нет)</t>
+        </is>
+      </c>
+      <c r="L10" s="14" t="inlineStr">
+        <is>
           <t>5-шаговый процесс: решение руководителя ОКК/директора по качеству (Акт забраковки ТМЦ, форма 03-01); действия сотрудника ОКК (письмо, Акт разрешения на отклонение, Журнал форма 03-03); отдельная ветка для опасного брака/аллергенов; роли ведущего технолога ПО/НА/ОИМРП/начальника ЛР; хранение и дальнейшие действия по браку.</t>
         </is>
       </c>
-      <c r="L10" s="14" t="inlineStr">
+      <c r="M10" s="14" t="inlineStr">
         <is>
           <t>ПР-03-00-12.doc — 62%; ПР-08-00-14 упомянут в тексте.</t>
         </is>
       </c>
-      <c r="M10" s="32" t="inlineStr">
+      <c r="N10" s="32" t="inlineStr">
         <is>
           <t>БЕЗ ИЗМЕНЕНИЙ (было верно, осталось верно) — ответ даже детальнее исходного (названы конкретные формы 03-01/03-03 и роли, которых не было в версии от 11.09)</t>
+        </is>
+      </c>
+      <c r="O10" s="37" t="inlineStr">
+        <is>
+          <t>Без изменений — верно</t>
         </is>
       </c>
     </row>
@@ -1021,17 +1161,27 @@
       </c>
       <c r="K11" s="14" t="inlineStr">
         <is>
+          <t>13:44–13:46 (единый диапазон по скриншоту условий теста; отдельных отметок времени на вопрос нет)</t>
+        </is>
+      </c>
+      <c r="L11" s="14" t="inlineStr">
+        <is>
           <t>В доступных источниках марка стретч-плёнки для обмотки паллет с готовой продукцией не указана. Найденный фрагмент Д-09-01-17 «План контроля тары и упаковки» содержит требования к пакетам и этикеткам, но не к стретч-плёнке.</t>
         </is>
       </c>
-      <c r="L11" s="14" t="inlineStr">
+      <c r="M11" s="14" t="inlineStr">
         <is>
           <t>Д-09-01-17 План контроля тары и упаковки.docx — 50%</t>
         </is>
       </c>
-      <c r="M11" s="32" t="inlineStr">
+      <c r="N11" s="32" t="inlineStr">
         <is>
           <t>БЕЗ ИЗМЕНЕНИЙ — верный ответ «не найдено» (уже подтверждено в pilot-test-01-analysis.md §5: марки в корпусе действительно нет)</t>
+        </is>
+      </c>
+      <c r="O11" s="37" t="inlineStr">
+        <is>
+          <t>Без изменений — верно</t>
         </is>
       </c>
     </row>
@@ -1069,17 +1219,27 @@
       </c>
       <c r="K12" s="14" t="inlineStr">
         <is>
+          <t>13:44–13:46 (единый диапазон по скриншоту условий теста; отдельных отметок времени на вопрос нет)</t>
+        </is>
+      </c>
+      <c r="L12" s="14" t="inlineStr">
+        <is>
           <t>В доступных источниках периодичность оценки квалификации внештатных сотрудников, работающих по договору подряда, не указана. В ПР-14-00-12 «Компетентность персонала» найдено поле «Оценка результативности», но срок или частота такой оценки не приведены.</t>
         </is>
       </c>
-      <c r="L12" s="14" t="inlineStr">
+      <c r="M12" s="14" t="inlineStr">
         <is>
           <t>Д-17-12-03 Оборудование для мониторинга и измерений.docx — 48%; ПР-14-00-12 Компетентность персонала.doc — 48%</t>
         </is>
       </c>
-      <c r="M12" s="32" t="inlineStr">
+      <c r="N12" s="32" t="inlineStr">
         <is>
           <t>БЕЗ ИЗМЕНЕНИЙ — вопрос остаётся открытым (был не подтверждён ни как ошибка, ни как верный ответ в pilot-test-01-analysis.md §5). Теперь хотя бы нашли релевантное поле «Оценка результативности» в ПР-14-00-12, но конкретики по подрядчикам по-прежнему нет — похоже, нужного документа/раздела действительно нет в корпусе.</t>
+        </is>
+      </c>
+      <c r="O12" s="38" t="inlineStr">
+        <is>
+          <t>Без изменений — открытый вопрос</t>
         </is>
       </c>
     </row>
@@ -1117,17 +1277,27 @@
       </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
+          <t>13:44–13:46 (единый диапазон по скриншоту условий теста; отдельных отметок времени на вопрос нет)</t>
+        </is>
+      </c>
+      <c r="L13" s="14" t="inlineStr">
+        <is>
           <t>В найденных источниках точный перечень полей журнала «Учёт уборки производственного оборудования», форма 17-08, не указан. Найден только перечень полей для журнала оборудования для мониторинга и измерений (другая форма): наименование оборудования и номер, дата последней поверки, подпись ответственного, дата следующей поверки, подпись ответственного, место установки, примечание.</t>
         </is>
       </c>
-      <c r="L13" s="14" t="inlineStr">
+      <c r="M13" s="14" t="inlineStr">
         <is>
           <t>Д-17-12-03 «Оборудование для мониторинга и измерений».docx — 75% (другой документ, не тот, что цитировался в пилоте — но вывод тот же: нужного перечня нет)</t>
         </is>
       </c>
-      <c r="M13" s="32" t="inlineStr">
+      <c r="N13" s="32" t="inlineStr">
         <is>
           <t>БЕЗ ИЗМЕНЕНИЙ — верный ответ «не найдено» (Форма 17-08 как бланк по-прежнему не в корпусе, см. pilot-test-01-analysis.md §5). Источник цитирования сменился на другой документ — не тот, что раньше, но конечный вывод не изменился.</t>
+        </is>
+      </c>
+      <c r="O13" s="37" t="inlineStr">
+        <is>
+          <t>Без изменений — верно</t>
         </is>
       </c>
     </row>
@@ -1165,17 +1335,27 @@
       </c>
       <c r="K14" s="34" t="inlineStr">
         <is>
+          <t>13:44–13:46 (единый диапазон по скриншоту условий теста; отдельных отметок времени на вопрос нет)</t>
+        </is>
+      </c>
+      <c r="L14" s="34" t="inlineStr">
+        <is>
           <t>1. Дождитесь уведомления ОКК о соответствии сырья требованиям. 2. ОКК направляет письмо руководителю ОКК, бухгалтерии, начальнику СО и оператору склада с просьбой переместить сырьё на соответствующий склад. 3. После перемещения на рабочий склад согласуйте с мастером ПО приоритетность задач. 4. В 1С8 во вкладке «Процесс» заказа установите флажок «Передать сырьё» и нажмите «Выгрузить WMS». 5. После выдачи оператор ПО забирает сырьё и доставляет к указанному аппарату.</t>
         </is>
       </c>
-      <c r="L14" s="34" t="inlineStr">
+      <c r="M14" s="34" t="inlineStr">
         <is>
           <t>ПР-09-00-14 «Контроль качества».doc — 49%; ПР-03-00-12.doc — 65%; Д-08-07-01 упомянут в тексте</t>
         </is>
       </c>
-      <c r="M14" s="34" t="inlineStr">
+      <c r="N14" s="34" t="inlineStr">
         <is>
           <t>УЛУЧШЕНО — раньше был открытый вопрос («прямого порядка... нет»), теперь дан полный прямой пошаговый ответ именно для склада «Проверка ОКК», с конкретным источником (ПР-09-00-14), который мы раньше не связывали с этим вопросом</t>
+        </is>
+      </c>
+      <c r="O14" s="34" t="inlineStr">
+        <is>
+          <t>Улучшено</t>
         </is>
       </c>
     </row>
@@ -1213,17 +1393,27 @@
       </c>
       <c r="K15" s="33" t="inlineStr">
         <is>
+          <t>13:44–13:46 (единый диапазон по скриншоту условий теста; отдельных отметок времени на вопрос нет)</t>
+        </is>
+      </c>
+      <c r="L15" s="33" t="inlineStr">
+        <is>
           <t>В доступных источниках не найден порядок приоритизации нескольких срочных заявок на ремонт. Поэтому определить, какую заявку выполнять первой, по имеющимся данным нельзя.</t>
         </is>
       </c>
-      <c r="L15" s="33" t="inlineStr">
+      <c r="M15" s="33" t="inlineStr">
         <is>
           <t>Источник не показан вообще (карточка «Ответ основан на источниках» отсутствует в ответе)</t>
         </is>
       </c>
-      <c r="M15" s="33" t="inlineStr">
+      <c r="N15" s="33" t="inlineStr">
         <is>
           <t>БЕЗ ИЗМЕНЕНИЙ — важное подтверждение гипотезы «Корневая причина №2» из proverka-zdorovya-zagruzki-predlozhenie.md: это retrieval-ошибка, не парсинг (источник ПР-10(02)-00.docx читаемый, ответ в нём есть текстом), и правки, починившие 1.2/1.3, её не задели — ровно как предсказывалось</t>
+        </is>
+      </c>
+      <c r="O15" s="35" t="inlineStr">
+        <is>
+          <t>Без изменений — ошибка сохраняется</t>
         </is>
       </c>
     </row>
@@ -1261,17 +1451,27 @@
       </c>
       <c r="K16" s="14" t="inlineStr">
         <is>
+          <t>13:44–13:46 (единый диапазон по скриншоту условий теста; отдельных отметок времени на вопрос нет)</t>
+        </is>
+      </c>
+      <c r="L16" s="14" t="inlineStr">
+        <is>
           <t>Срочный заказ покупателя имеет приоритет над наработкой продукции на склад (если у заказа нет поля «Приоритет» или указан «0», выполняется после заказов «1»/«2»). Порядок: 1) через отчёт «Загруженность оборудования» определить окно; 2) согласовать график наработки с мастером ПО/техдиректором/начальником ПУ; 3) сформировать заказ на производство на доп. объём без привязки к заказу покупателя; 4) проверить складские остатки аналогичной продукции.</t>
         </is>
       </c>
-      <c r="L16" s="14" t="inlineStr">
+      <c r="M16" s="14" t="inlineStr">
         <is>
           <t>И-12-10-03.docx 63%; ПР-08-00-14.doc 49%; Д-08-03-01.doc 49%; И-08-08-01.docx 48% — все релевантны, аномалий нет</t>
         </is>
       </c>
-      <c r="M16" s="32" t="inlineStr">
+      <c r="N16" s="32" t="inlineStr">
         <is>
           <t>БЕЗ ИЗМЕНЕНИЙ (было верно, осталось верно) — не входил в число ошибок пилота; ответ даже детальнее, с постатейной сверкой источников</t>
+        </is>
+      </c>
+      <c r="O16" s="37" t="inlineStr">
+        <is>
+          <t>Без изменений — верно</t>
         </is>
       </c>
     </row>
@@ -1309,17 +1509,27 @@
       </c>
       <c r="K17" s="14" t="inlineStr">
         <is>
+          <t>13:44–13:46 (единый диапазон по скриншоту условий теста; отдельных отметок времени на вопрос нет)</t>
+        </is>
+      </c>
+      <c r="L17" s="14" t="inlineStr">
+        <is>
           <t>1. Перед началом проверяет в Рабочей инструкции на производство (форма 16-03): примечания к технологическому процессу, вид фасовки. 2. Осматривает тару и упаковку. 3. Выполняет фасовку по И-08-02 «Фасовка и упаковка готовой продукции». 4. После каждого этапа — запись и подпись. 5. Вывозит продукцию в зону передачи на склад. 6. Передаёт заполненную рабочую инструкцию ответственному сотруднику ПО. Фасовке подлежит продукция с положительным заключением ОКК либо продукция, предназначенная для перефасовки.</t>
         </is>
       </c>
-      <c r="L17" s="14" t="inlineStr">
+      <c r="M17" s="14" t="inlineStr">
         <is>
           <t>ПР-08-00-14 «Производственный процесс», разделы 5.4-5.7.doc — 57%; И-08-02-10 «Фасовка и упаковка готовой продукции».doc — 50%</t>
         </is>
       </c>
-      <c r="M17" s="32" t="inlineStr">
+      <c r="N17" s="32" t="inlineStr">
         <is>
           <t>БЕЗ ИЗМЕНЕНИЙ (было верно, осталось верно) — не входил в число ошибок пилота, ответ детальнее исходного</t>
+        </is>
+      </c>
+      <c r="O17" s="37" t="inlineStr">
+        <is>
+          <t>Без изменений — верно</t>
         </is>
       </c>
     </row>
@@ -1357,17 +1567,27 @@
       </c>
       <c r="K18" s="35" t="inlineStr">
         <is>
+          <t>13:44–13:46 (единый диапазон по скриншоту условий теста; отдельных отметок времени на вопрос нет)</t>
+        </is>
+      </c>
+      <c r="L18" s="35" t="inlineStr">
+        <is>
           <t>ОШИБКА СЕРВИСА (дважды подряд, 13:50 и 13:51): «Не удалось получить ответ модели (временная ошибка сервиса). Попробуйте повторить запрос или переформулировать короче.» Содержательного ответа нет ни разу.</t>
         </is>
       </c>
-      <c r="L18" s="35" t="inlineStr">
+      <c r="M18" s="35" t="inlineStr">
         <is>
           <t>Даже при отказе модели показаны источники — но НЕ те: Д-08-03-01 «Формирование заказов на производство» (63-64%) и Д-08-04-01 «Проведение корректировок к заказу на производство» (59-61%). Ни разу не показан И-08-05-08 «Внесение спецификаций в базе 1С-8» — реальный нужный источник по разбору ошибок пилота.</t>
         </is>
       </c>
-      <c r="M18" s="35" t="inlineStr">
+      <c r="N18" s="35" t="inlineStr">
         <is>
           <t>НЕ ОЦЕНИВАЕТСЯ — служебная ошибка модели, а не содержательный ответ. Отдельно тревожно: retrieval даже не подтягивает нужный документ (И-08-05-08) — похоже на путаницу с похожими по теме документами «заказ на производство», а не на восстановленный/сломанный формат</t>
+        </is>
+      </c>
+      <c r="O18" s="39" t="inlineStr">
+        <is>
+          <t>Не оценивается (служебная ошибка)</t>
         </is>
       </c>
     </row>
@@ -1405,17 +1625,27 @@
       </c>
       <c r="K19" s="14" t="inlineStr">
         <is>
+          <t>13:44–13:46 (единый диапазон по скриншоту условий теста; отдельных отметок времени на вопрос нет)</t>
+        </is>
+      </c>
+      <c r="L19" s="14" t="inlineStr">
+        <is>
           <t>Процесс установлен документом ПР-09-00 «Контроль качества»: 1) контроль на складе сырья СО или в ОКК; 2) результаты в журнал «Контроль сырья и первичной упаковки» (форма 09-01) с полным перечнем полей; 3) при несоответствии решение принимает руководитель ОКК/директор по качеству; 4) оформляются Акт забраковки (03-01)/Акт разрешения на отклонение (03-02)/Акт на утилизацию (03-04), запись в журнал 03-03; 5) решение о применении сырья и коррекции — руководитель/директор по качеству.</t>
         </is>
       </c>
-      <c r="L19" s="14" t="inlineStr">
+      <c r="M19" s="14" t="inlineStr">
         <is>
           <t>ПР-09-00-14 «Контроль качества».doc — 63%; ПР-03-00-12 упомянут в тексте</t>
         </is>
       </c>
-      <c r="M19" s="32" t="inlineStr">
+      <c r="N19" s="32" t="inlineStr">
         <is>
           <t>БЕЗ ИЗМЕНЕНИЙ (было верно, осталось верно) — не входил в число ошибок пилота, ответ детальнее исходного (конкретные формы 09-01/03-01/03-02/03-03/03-04)</t>
+        </is>
+      </c>
+      <c r="O19" s="37" t="inlineStr">
+        <is>
+          <t>Без изменений — верно</t>
         </is>
       </c>
     </row>

</xml_diff>